<commit_message>
feat(pos_sync): rapikan handover Krim Kopi jadi 1 MR bulk per hari
</commit_message>
<xml_diff>
--- a/pos_sync/Laporan_Bersih_Dokumen_Cancelled.xlsx
+++ b/pos_sync/Laporan_Bersih_Dokumen_Cancelled.xlsx
@@ -454,10 +454,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C2" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,12 +494,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Stock Entry</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SE-MR-261009001-1</t>
+          <t>MREQ-MTR-26-0190</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -511,12 +511,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Stock Entry</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SE-MR-261009001</t>
+          <t>MREQ-MTR-26-0193</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -528,12 +528,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Stock Entry</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SE-MR-261009002</t>
+          <t>MREQ-MTR-26-0194</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -545,12 +545,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Purchase Receipt</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PR-061026-011</t>
+          <t>MREQ-MTR-26-0195</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -562,12 +562,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Purchase Receipt</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PR-061026-012</t>
+          <t>MREQ-MTR-26-0196</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -579,12 +579,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Purchase Receipt</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PR-061026-014</t>
+          <t>MREQ-MTR-26-0197</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -596,12 +596,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Purchase Receipt</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PR-061026-017-OLD</t>
+          <t>MREQ-MTR-26-0198</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -613,12 +613,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Purchase Invoice</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PI-JURI-261008005</t>
+          <t>MREQ-MTR-26-0199</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -630,12 +630,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Purchase Invoice</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PI-JURI-261008006</t>
+          <t>MREQ-MTR-26-0200</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -647,12 +647,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Purchase Invoice</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PI-JURI-261008011</t>
+          <t>MREQ-MTR-26-0201</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -664,12 +664,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Delivery Note</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DN-011026-026</t>
+          <t>MREQ-MTR-26-0202</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -681,12 +681,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Delivery Note</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DN-021026-010</t>
+          <t>MREQ-MTR-26-0203</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -698,12 +698,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Delivery Note</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DN-061026-003</t>
+          <t>MREQ-MTR-26-0204</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -715,12 +715,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Stock Reconciliation</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>RECO-JURI-261006004</t>
+          <t>MREQ-MTR-26-0205</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -732,12 +732,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Stock Reconciliation</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RECO-JURI-261007004</t>
+          <t>MREQ-MTR-26-0206</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -749,12 +749,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Stock Reconciliation</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>RECO-JURI-261007005</t>
+          <t>MREQ-MTR-26-0207</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -766,12 +766,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Stock Reconciliation</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>RECO-JURI-261007006</t>
+          <t>MREQ-MTR-26-0208</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -783,12 +783,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Stock Reconciliation</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>RECO-JURI-261008002</t>
+          <t>MREQ-MTR-26-0209</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -800,12 +800,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Stock Reconciliation</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>RECO-JURI-261009015</t>
+          <t>MREQ-MTR-26-0210</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -817,12 +817,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Stock Reconciliation</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>RECO-JURI-261009016</t>
+          <t>MREQ-MTR-26-0211</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -834,12 +834,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Stock Reconciliation</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>RECO-JURI-261009027</t>
+          <t>MREQ-MTR-26-0212</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -851,12 +851,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Stock Reconciliation</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>RECO-JURI-261009028</t>
+          <t>MREQ-MTR-26-0213</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -868,12 +868,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Purchase Order</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PO-021026-003</t>
+          <t>MREQ-MTR-26-0214</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -885,12 +885,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Purchase Order</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PO-021026-020</t>
+          <t>MREQ-MTR-26-0215</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -902,12 +902,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Purchase Order</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PO-021026-022</t>
+          <t>MREQ-MTR-26-0216</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -919,12 +919,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Purchase Order</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>PO-061026-005</t>
+          <t>MREQ-MTR-26-0217</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -936,12 +936,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Purchase Order</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PO-061026-006</t>
+          <t>MREQ-MTR-26-0218</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -953,12 +953,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Purchase Order</t>
+          <t>Material Request</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PO-061026-007</t>
+          <t>MREQ-MTR-26-0219</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MREQ-PUR-26-0059</t>
+          <t>MREQ-MTR-26-0220</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -992,10 +992,95 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MREQ-PUR-26-0060</t>
+          <t>MREQ-MTR-26-0221</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
+        <is>
+          <t>DELETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Material Request</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>MREQ-MTR-26-0222</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>DELETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Material Request</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>MREQ-MTR-26-0223</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>DELETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Material Request</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>MREQ-MTR-26-0224</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>DELETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Material Request</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>MREQ-MTR-26-0225</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>DELETED</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Material Request</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>MREQ-MTR-26-0226</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
         <is>
           <t>DELETED</t>
         </is>

</xml_diff>